<commit_message>
Reorganize sequence files into seqs_T1Rs and seqs_LPH subdirectories; update README and data files
</commit_message>
<xml_diff>
--- a/data/Fig2A_KEGG_David_Pipridae.xlsx
+++ b/data/Fig2A_KEGG_David_Pipridae.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10525"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mbp23/ownCloud/Baldwin/Projects/Manakin/Rscripts/for_github/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/meng-ching.ko/ownCloud/Baldwin/Projects/Manakin/Rscripts/for_github/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16154358-6F11-D049-9D17-DB668F0F33A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0BC0E08-56DD-F440-A07A-9B70F34F685B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1580" yWindow="5320" windowWidth="25600" windowHeight="17540" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1580" yWindow="1220" windowWidth="25600" windowHeight="17540" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
   <si>
     <t>Pipridae</t>
   </si>
@@ -36,18 +36,12 @@
     <t>hsa04974:Protein digestion and absorption</t>
   </si>
   <si>
-    <t>Many</t>
-  </si>
-  <si>
     <t>SLC9A3, COL3A1, COL15A1, CTRL, COL4A1, COL12A1, COL6A1, COL6A3, ATP1A1</t>
   </si>
   <si>
     <t>hsa04060:Cytokine-cytokine receptor interaction</t>
   </si>
   <si>
-    <t>Immune</t>
-  </si>
-  <si>
     <t>IL18RAP, IL20, IL12B, IL20RB, TNFRSF8, CCR7, IFNLR1, IL7R, IL12RB1, IL12RB2</t>
   </si>
   <si>
@@ -78,9 +72,6 @@
     <t>hsa04973:Carbohydrate digestion and absorption</t>
   </si>
   <si>
-    <t>Diet</t>
-  </si>
-  <si>
     <t>SI, ATP1A1, LCT, SLC2A5</t>
   </si>
   <si>
@@ -106,12 +97,6 @@
   </si>
   <si>
     <t>Term</t>
-  </si>
-  <si>
-    <t>Synthetic Category</t>
-  </si>
-  <si>
-    <t>Additional diet</t>
   </si>
   <si>
     <t>Count</t>
@@ -527,60 +512,54 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="32.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="B1" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>26</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>27</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>28</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>29</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>30</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>31</v>
       </c>
-      <c r="K1" t="s">
-        <v>32</v>
-      </c>
-      <c r="L1" t="s">
-        <v>33</v>
-      </c>
-      <c r="M1" t="s">
-        <v>34</v>
-      </c>
-      <c r="N1" t="s">
-        <v>35</v>
-      </c>
-      <c r="O1" t="s">
-        <v>36</v>
-      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -596,35 +575,32 @@
       <c r="E2" t="s">
         <v>2</v>
       </c>
-      <c r="G2" t="s">
+      <c r="F2">
+        <v>9</v>
+      </c>
+      <c r="G2" s="1">
+        <v>1.16546748829923E-4</v>
+      </c>
+      <c r="H2" t="s">
         <v>3</v>
       </c>
-      <c r="H2">
-        <v>9</v>
-      </c>
-      <c r="I2" s="1">
-        <v>1.16546748829923E-4</v>
-      </c>
-      <c r="J2" t="s">
-        <v>4</v>
+      <c r="I2">
+        <v>114</v>
+      </c>
+      <c r="J2">
+        <v>44</v>
       </c>
       <c r="K2">
-        <v>114</v>
+        <v>3196</v>
       </c>
       <c r="L2">
-        <v>44</v>
-      </c>
-      <c r="M2">
-        <v>3196</v>
-      </c>
-      <c r="N2">
         <v>5.7344497607655498</v>
       </c>
-      <c r="O2" s="2">
+      <c r="M2" s="2">
         <v>1.7789117091241199E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>5</v>
       </c>
@@ -638,37 +614,34 @@
         <v>1</v>
       </c>
       <c r="E3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>10</v>
+      </c>
+      <c r="G3">
+        <v>4.0049189437626597E-3</v>
+      </c>
+      <c r="H3" t="s">
         <v>5</v>
       </c>
-      <c r="F3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3">
-        <v>10</v>
-      </c>
       <c r="I3">
-        <v>4.0049189437626597E-3</v>
-      </c>
-      <c r="J3" t="s">
-        <v>7</v>
+        <v>114</v>
+      </c>
+      <c r="J3">
+        <v>90</v>
       </c>
       <c r="K3">
-        <v>114</v>
+        <v>3196</v>
       </c>
       <c r="L3">
-        <v>90</v>
+        <v>3.1150097465886901</v>
       </c>
       <c r="M3">
-        <v>3196</v>
-      </c>
-      <c r="N3">
-        <v>3.1150097465886901</v>
-      </c>
-      <c r="O3">
         <v>0.46097636357914701</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>6</v>
       </c>
@@ -682,34 +655,34 @@
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>8</v>
-      </c>
-      <c r="H4">
+        <v>6</v>
+      </c>
+      <c r="F4">
         <v>7</v>
       </c>
+      <c r="G4">
+        <v>1.31460838992305E-2</v>
+      </c>
+      <c r="H4" t="s">
+        <v>7</v>
+      </c>
       <c r="I4">
-        <v>1.31460838992305E-2</v>
-      </c>
-      <c r="J4" t="s">
-        <v>9</v>
+        <v>114</v>
+      </c>
+      <c r="J4">
+        <v>56</v>
       </c>
       <c r="K4">
-        <v>114</v>
+        <v>3196</v>
       </c>
       <c r="L4">
-        <v>56</v>
+        <v>3.5043859649122799</v>
       </c>
       <c r="M4">
-        <v>3196</v>
-      </c>
-      <c r="N4">
-        <v>3.5043859649122799</v>
-      </c>
-      <c r="O4">
         <v>0.86970078376550297</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>9</v>
       </c>
@@ -723,37 +696,34 @@
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H5">
+        <v>8</v>
+      </c>
+      <c r="F5">
         <v>5</v>
       </c>
+      <c r="G5">
+        <v>2.23175547893085E-2</v>
+      </c>
+      <c r="H5" t="s">
+        <v>9</v>
+      </c>
       <c r="I5">
-        <v>2.23175547893085E-2</v>
-      </c>
-      <c r="J5" t="s">
-        <v>11</v>
+        <v>114</v>
+      </c>
+      <c r="J5">
+        <v>31</v>
       </c>
       <c r="K5">
-        <v>114</v>
+        <v>3196</v>
       </c>
       <c r="L5">
-        <v>31</v>
+        <v>4.5217883418222904</v>
       </c>
       <c r="M5">
-        <v>3196</v>
-      </c>
-      <c r="N5">
-        <v>4.5217883418222904</v>
-      </c>
-      <c r="O5">
         <v>0.96906402128003299</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>10</v>
       </c>
@@ -767,34 +737,34 @@
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H6">
+        <v>10</v>
+      </c>
+      <c r="F6">
         <v>5</v>
       </c>
+      <c r="G6">
+        <v>2.4828280898176999E-2</v>
+      </c>
+      <c r="H6" t="s">
+        <v>11</v>
+      </c>
       <c r="I6">
-        <v>2.4828280898176999E-2</v>
-      </c>
-      <c r="J6" t="s">
-        <v>13</v>
+        <v>114</v>
+      </c>
+      <c r="J6">
+        <v>32</v>
       </c>
       <c r="K6">
-        <v>114</v>
+        <v>3196</v>
       </c>
       <c r="L6">
-        <v>32</v>
+        <v>4.3804824561403501</v>
       </c>
       <c r="M6">
-        <v>3196</v>
-      </c>
-      <c r="N6">
-        <v>4.3804824561403501</v>
-      </c>
-      <c r="O6">
         <v>0.97917960004372295</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>14</v>
       </c>
@@ -808,34 +778,34 @@
         <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7">
+        <v>12</v>
+      </c>
+      <c r="F7">
         <v>7</v>
       </c>
+      <c r="G7">
+        <v>3.5680771278666201E-2</v>
+      </c>
+      <c r="H7" t="s">
+        <v>13</v>
+      </c>
       <c r="I7">
-        <v>3.5680771278666201E-2</v>
-      </c>
-      <c r="J7" t="s">
-        <v>15</v>
+        <v>114</v>
+      </c>
+      <c r="J7">
+        <v>70</v>
       </c>
       <c r="K7">
-        <v>114</v>
+        <v>3196</v>
       </c>
       <c r="L7">
-        <v>70</v>
+        <v>2.80350877192982</v>
       </c>
       <c r="M7">
-        <v>3196</v>
-      </c>
-      <c r="N7">
-        <v>2.80350877192982</v>
-      </c>
-      <c r="O7">
         <v>0.99628458506711803</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>15</v>
       </c>
@@ -849,37 +819,34 @@
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8">
+        <v>14</v>
+      </c>
+      <c r="F8">
         <v>4</v>
       </c>
+      <c r="G8">
+        <v>3.5992872672372701E-2</v>
+      </c>
+      <c r="H8" t="s">
+        <v>15</v>
+      </c>
       <c r="I8">
-        <v>3.5992872672372701E-2</v>
-      </c>
-      <c r="J8" t="s">
-        <v>18</v>
+        <v>114</v>
+      </c>
+      <c r="J8">
+        <v>21</v>
       </c>
       <c r="K8">
-        <v>114</v>
+        <v>3196</v>
       </c>
       <c r="L8">
-        <v>21</v>
+        <v>5.3400167084377603</v>
       </c>
       <c r="M8">
-        <v>3196</v>
-      </c>
-      <c r="N8">
-        <v>5.3400167084377603</v>
-      </c>
-      <c r="O8">
         <v>0.99646525811563402</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>25</v>
       </c>
@@ -893,37 +860,34 @@
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" t="s">
-        <v>6</v>
-      </c>
-      <c r="H9">
+        <v>16</v>
+      </c>
+      <c r="F9">
         <v>4</v>
       </c>
+      <c r="G9">
+        <v>6.1998589031891302E-2</v>
+      </c>
+      <c r="H9" t="s">
+        <v>17</v>
+      </c>
       <c r="I9">
-        <v>6.1998589031891302E-2</v>
-      </c>
-      <c r="J9" t="s">
-        <v>20</v>
+        <v>114</v>
+      </c>
+      <c r="J9">
+        <v>26</v>
       </c>
       <c r="K9">
-        <v>114</v>
+        <v>3196</v>
       </c>
       <c r="L9">
-        <v>26</v>
+        <v>4.3130904183535703</v>
       </c>
       <c r="M9">
-        <v>3196</v>
-      </c>
-      <c r="N9">
-        <v>4.3130904183535703</v>
-      </c>
-      <c r="O9">
         <v>0.99994759922438703</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>26</v>
       </c>
@@ -937,30 +901,30 @@
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>21</v>
-      </c>
-      <c r="H10">
+        <v>18</v>
+      </c>
+      <c r="F10">
         <v>9</v>
       </c>
+      <c r="G10">
+        <v>6.4654544838208802E-2</v>
+      </c>
+      <c r="H10" t="s">
+        <v>19</v>
+      </c>
       <c r="I10">
-        <v>6.4654544838208802E-2</v>
-      </c>
-      <c r="J10" t="s">
-        <v>22</v>
+        <v>114</v>
+      </c>
+      <c r="J10">
+        <v>122</v>
       </c>
       <c r="K10">
-        <v>114</v>
+        <v>3196</v>
       </c>
       <c r="L10">
-        <v>122</v>
+        <v>2.0681622088006901</v>
       </c>
       <c r="M10">
-        <v>3196</v>
-      </c>
-      <c r="N10">
-        <v>2.0681622088006901</v>
-      </c>
-      <c r="O10">
         <v>0.99996613943395296</v>
       </c>
     </row>

</xml_diff>